<commit_message>
feat(roadmap): hito Encendido como punto verde en el timeline
</commit_message>
<xml_diff>
--- a/public/matriz_backlog.xlsx
+++ b/public/matriz_backlog.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30619"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/miguelangelpacheco/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{01119B08-5E1A-490C-8A79-59D2A15C27E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{956455F2-5413-4288-AE4C-8ADEDB2F2C85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16980" xr2:uid="{F5EBCA54-F250-EF45-B6B3-60EFDB3A97A7}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Proyectos - Nego - Regu" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Proyectos - Nego - Regu'!$A$1:$Q$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Proyectos - Nego - Regu'!$A$1:$Q$49</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>

</xml_diff>